<commit_message>
[codex] art: wire V2 HUD and workbench assets
</commit_message>
<xml_diff>
--- a/아트-발주서.xlsx
+++ b/아트-발주서.xlsx
@@ -851,40 +851,40 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="0">
+      <c r="A20" s="2">
         <v>3</v>
       </c>
-      <c r="B20" s="0" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">배경</t>
         </is>
       </c>
-      <c r="C20" s="0" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg/autopsy.png</t>
         </is>
       </c>
-      <c r="D20" s="0" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1920×936</t>
         </is>
       </c>
-      <c r="E20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F20" s="0" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">⑤ 검시실</t>
         </is>
       </c>
-      <c r="G20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H20" s="0" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg.autopsy</t>
         </is>
@@ -931,40 +931,40 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="0">
+      <c r="A22" s="2">
         <v>3</v>
       </c>
-      <c r="B22" s="0" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">배경</t>
         </is>
       </c>
-      <c r="C22" s="0" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg/live.png</t>
         </is>
       </c>
-      <c r="D22" s="0" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1920×1080</t>
         </is>
       </c>
-      <c r="E22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F22" s="0" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">③ 생방송 5분할 바탕 (칸 사이 여백)</t>
         </is>
       </c>
-      <c r="G22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H22" s="0" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg.live</t>
         </is>
@@ -1051,40 +1051,40 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="0">
+      <c r="A25" s="2">
         <v>3</v>
       </c>
-      <c r="B25" s="0" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">배경</t>
         </is>
       </c>
-      <c r="C25" s="0" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg/studio.png</t>
         </is>
       </c>
-      <c r="D25" s="0" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1920×936</t>
         </is>
       </c>
-      <c r="E25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F25" s="0" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">⑥ 발표 스튜디오</t>
         </is>
       </c>
-      <c r="G25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H25" s="0" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bg.studio</t>
         </is>
@@ -1491,40 +1491,40 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="0">
+      <c r="A36" s="2">
         <v>3</v>
       </c>
-      <c r="B36" s="0" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">UI · 버튼</t>
         </is>
       </c>
-      <c r="C36" s="0" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui/button_danger.png</t>
         </is>
       </c>
-      <c r="D36" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32×32</t>
-        </is>
-      </c>
-      <c r="E36" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
-        </is>
-      </c>
-      <c r="F36" s="0" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">208×88</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">버튼 크기에 맞춰 늘어난다 (모서리 22px 고정)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버튼 위험 (소생·어필·훼손)</t>
         </is>
       </c>
-      <c r="G36" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H36" s="0" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui.button.danger.9s</t>
         </is>
@@ -1546,12 +1546,12 @@
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">32×32</t>
+          <t xml:space="preserve">208×88</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
+          <t xml:space="preserve">버튼 크기에 맞춰 늘어난다 (모서리 22px 고정)</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
@@ -1571,80 +1571,80 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="0">
+      <c r="A38" s="2">
         <v>3</v>
       </c>
-      <c r="B38" s="0" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">UI · 버튼</t>
         </is>
       </c>
-      <c r="C38" s="0" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui/button_hover.png</t>
         </is>
       </c>
-      <c r="D38" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32×32</t>
-        </is>
-      </c>
-      <c r="E38" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
-        </is>
-      </c>
-      <c r="F38" s="0" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">208×88</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">버튼 크기에 맞춰 늘어난다 (모서리 22px 고정)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버튼 마우스오버</t>
         </is>
       </c>
-      <c r="G38" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H38" s="0" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui.button.hover.9s</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="0">
+      <c r="A39" s="2">
         <v>3</v>
       </c>
-      <c r="B39" s="0" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">UI · 버튼</t>
         </is>
       </c>
-      <c r="C39" s="0" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui/button.png</t>
         </is>
       </c>
-      <c r="D39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32×32</t>
-        </is>
-      </c>
-      <c r="E39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
-        </is>
-      </c>
-      <c r="F39" s="0" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">208×88</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">버튼 크기에 맞춰 늘어난다 (모서리 22px 고정)</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버튼 평상</t>
         </is>
       </c>
-      <c r="G39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H39" s="0" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ui.button.9s</t>
         </is>
@@ -1971,200 +1971,200 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="0">
-        <v>4</v>
-      </c>
-      <c r="B48" s="0" t="inlineStr">
+      <c r="A48" s="2">
+        <v>4</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">소품</t>
         </is>
       </c>
-      <c r="C48" s="0" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop/lamp.png</t>
         </is>
       </c>
-      <c r="D48" s="0" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">224×352</t>
         </is>
       </c>
-      <c r="E48" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F48" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">작업대 램프 (광원)</t>
-        </is>
-      </c>
-      <c r="G48" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H48" s="0" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">작업대의 실제 석유 램프</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop.lamp</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="0">
-        <v>4</v>
-      </c>
-      <c r="B49" s="0" t="inlineStr">
+      <c r="A49" s="2">
+        <v>4</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">소품</t>
         </is>
       </c>
-      <c r="C49" s="0" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop/ledger.png</t>
         </is>
       </c>
-      <c r="D49" s="0" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">336×264</t>
         </is>
       </c>
-      <c r="E49" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F49" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">장부</t>
-        </is>
-      </c>
-      <c r="G49" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H49" s="0" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">작업대의 출연자 서류철</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop.ledger</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="0">
-        <v>4</v>
-      </c>
-      <c r="B50" s="0" t="inlineStr">
+      <c r="A50" s="2">
+        <v>4</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">소품</t>
         </is>
       </c>
-      <c r="C50" s="0" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop/scroll.png</t>
         </is>
       </c>
-      <c r="D50" s="0" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">176×64</t>
         </is>
       </c>
-      <c r="E50" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F50" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">두루마리</t>
-        </is>
-      </c>
-      <c r="G50" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H50" s="0" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">계약서 서류 조각</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop.scroll</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="0">
-        <v>4</v>
-      </c>
-      <c r="B51" s="0" t="inlineStr">
+      <c r="A51" s="2">
+        <v>4</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">소품</t>
         </is>
       </c>
-      <c r="C51" s="0" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop/stamp.png</t>
         </is>
       </c>
-      <c r="D51" s="0" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">128×208</t>
         </is>
       </c>
-      <c r="E51" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F51" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">도장</t>
-        </is>
-      </c>
-      <c r="G51" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H51" s="0" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">최종 판정서에서 잘라낸 실물 도장</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop.stamp</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="0">
-        <v>4</v>
-      </c>
-      <c r="B52" s="0" t="inlineStr">
+      <c r="A52" s="2">
+        <v>4</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">소품</t>
         </is>
       </c>
-      <c r="C52" s="0" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop/tag.png</t>
         </is>
       </c>
-      <c r="D52" s="0" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">152×104</t>
         </is>
       </c>
-      <c r="E52" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F52" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가격표</t>
-        </is>
-      </c>
-      <c r="G52" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H52" s="0" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">작업대의 가격표</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">prop.tag</t>
         </is>
@@ -2251,82 +2251,82 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="0">
-        <v>4</v>
-      </c>
-      <c r="B55" s="0" t="inlineStr">
+      <c r="A55" s="2">
+        <v>4</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">UI · 기타</t>
         </is>
       </c>
-      <c r="C55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui/logo.png</t>
-        </is>
-      </c>
-      <c r="D55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">960×240</t>
-        </is>
-      </c>
-      <c r="E55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1:1</t>
-        </is>
-      </c>
-      <c r="F55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">타이틀 로고</t>
-        </is>
-      </c>
-      <c r="G55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H55" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui.logo</t>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/hud_status.png</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">700×144</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상단바 좌 — DAY·골드·팬·평판 4칸</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.hud.status</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="0">
-        <v>4</v>
-      </c>
-      <c r="B56" s="0" t="inlineStr">
+      <c r="A56" s="2">
+        <v>4</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">UI · 기타</t>
         </is>
       </c>
-      <c r="C56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui/seal.png</t>
-        </is>
-      </c>
-      <c r="D56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">768×192</t>
-        </is>
-      </c>
-      <c r="E56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">192×192 프레임 1칸 (1:1)</t>
-        </is>
-      </c>
-      <c r="F56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">봉랍 도장 4프레임</t>
-        </is>
-      </c>
-      <c r="G56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui.seal</t>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/hud_tools.png</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">740×144</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상단바 우 — 시계·도달층 게이지</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.hud.tools</t>
         </is>
       </c>
     </row>
@@ -2341,12 +2341,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/suspicion1.png</t>
+          <t xml:space="preserve">ui/icon_help_hover.png</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">192×128</t>
+          <t xml:space="preserve">112×112</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">의심도 1/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+          <t xml:space="preserve">상단바 아이콘 · 조작 안내(책) (눌림)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui.suspicion1</t>
+          <t xml:space="preserve">ui.icon.help.hover</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2381,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/suspicion2.png</t>
+          <t xml:space="preserve">ui/icon_help.png</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">192×128</t>
+          <t xml:space="preserve">112×112</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">의심도 2/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+          <t xml:space="preserve">상단바 아이콘 · 조작 안내(책)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui.suspicion2</t>
+          <t xml:space="preserve">ui.icon.help</t>
         </is>
       </c>
     </row>
@@ -2421,12 +2421,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/suspicion3.png</t>
+          <t xml:space="preserve">ui/icon_options_hover.png</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">192×128</t>
+          <t xml:space="preserve">112×112</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">의심도 3/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+          <t xml:space="preserve">상단바 아이콘 · 옵션(톱니) (눌림)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui.suspicion3</t>
+          <t xml:space="preserve">ui.icon.options.hover</t>
         </is>
       </c>
     </row>
@@ -2461,12 +2461,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/suspicion4.png</t>
+          <t xml:space="preserve">ui/icon_options.png</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">192×128</t>
+          <t xml:space="preserve">112×112</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">의심도 4/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+          <t xml:space="preserve">상단바 아이콘 · 옵션(톱니)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui.suspicion4</t>
+          <t xml:space="preserve">ui.icon.options</t>
         </is>
       </c>
     </row>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/suspicion5.png</t>
+          <t xml:space="preserve">ui/icon_save_hover.png</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">192×128</t>
+          <t xml:space="preserve">112×112</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">의심도 5/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+          <t xml:space="preserve">상단바 아이콘 · 저장 (눌림)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -2526,47 +2526,47 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui.suspicion5</t>
+          <t xml:space="preserve">ui.icon.save.hover</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="0">
-        <v>4</v>
-      </c>
-      <c r="B62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UI · 패널</t>
-        </is>
-      </c>
-      <c r="C62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui/panel_sunken.png</t>
-        </is>
-      </c>
-      <c r="D62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">48×48</t>
-        </is>
-      </c>
-      <c r="E62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
-        </is>
-      </c>
-      <c r="F62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">패널 테두리 (함몰 · 목록/채팅창)</t>
-        </is>
-      </c>
-      <c r="G62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">대기</t>
-        </is>
-      </c>
-      <c r="H62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ui.panel.sunken.9s</t>
+      <c r="A62" s="2">
+        <v>4</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/icon_save.png</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">112×112</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상단바 아이콘 · 저장</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.icon.save</t>
         </is>
       </c>
     </row>
@@ -2576,41 +2576,361 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/logo.png</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">960×240</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">타이틀 로고</t>
+        </is>
+      </c>
+      <c r="G63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대기</t>
+        </is>
+      </c>
+      <c r="H63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.logo</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0">
+        <v>4</v>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/seal.png</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">768×192</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×192 프레임 1칸 (1:1)</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">봉랍 도장 4프레임</t>
+        </is>
+      </c>
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대기</t>
+        </is>
+      </c>
+      <c r="H64" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.seal</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2">
+        <v>4</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/suspicion1.png</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×128</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의심도 1/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.suspicion1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2">
+        <v>4</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/suspicion2.png</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×128</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의심도 2/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.suspicion2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2">
+        <v>4</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/suspicion3.png</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×128</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의심도 3/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.suspicion3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2">
+        <v>4</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/suspicion4.png</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×128</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의심도 4/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.suspicion4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2">
+        <v>4</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 기타</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/suspicion5.png</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">192×128</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의심도 5/5 — 눈이 떠지는 5단 (5장 다 있어야 승계 화면에 뜬다)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도착</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.suspicion5</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0">
+        <v>4</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">UI · 패널</t>
         </is>
       </c>
-      <c r="C63" s="0" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/panel_sunken.png</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48×48</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">패널 테두리 (함몰 · 목록/채팅창)</t>
+        </is>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대기</t>
+        </is>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui.panel.sunken.9s</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0">
+        <v>4</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI · 패널</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">ui/panel.png</t>
         </is>
       </c>
-      <c r="D63" s="0" t="inlineStr">
+      <c r="D71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">48×48</t>
         </is>
       </c>
-      <c r="E63" s="0" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">버튼/패널 크기에 맞춰 늘어난다</t>
         </is>
       </c>
-      <c r="F63" s="0" t="inlineStr">
+      <c r="F71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">패널 테두리 (융기)</t>
         </is>
       </c>
-      <c r="G63" s="0" t="inlineStr">
+      <c r="G71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">대기</t>
         </is>
       </c>
-      <c r="H63" s="0" t="inlineStr">
+      <c r="H71" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">ui.panel.9s</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H63"/>
+  <autoFilter ref="A1:H71"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[codex] art: preserve source aspect in screen layouts
</commit_message>
<xml_diff>
--- a/아트-발주서.xlsx
+++ b/아트-발주서.xlsx
@@ -346,7 +346,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1152×792</t>
+          <t xml:space="preserve">1244×792</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -386,7 +386,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">752×792</t>
+          <t xml:space="preserve">650×792</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -426,7 +426,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">744×720</t>
+          <t xml:space="preserve">1000×792</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">

</xml_diff>